<commit_message>
Daily NSE scan: 2026-09-21
</commit_message>
<xml_diff>
--- a/output/2026-09-21/enriched_analysis.xlsx
+++ b/output/2026-09-21/enriched_analysis.xlsx
@@ -7573,12 +7573,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>VIVIANA</t>
+          <t>NPST</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>VIVIANA POWER TECH LIMITED</t>
+          <t>NETWORK PEOPLE SERVICES TECHNOLOGIES LIMITED</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -7590,185 +7590,187 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="F31" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G31" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="H31" t="n">
-        <v>0</v>
+        <v>-16</v>
       </c>
       <c r="I31" t="n">
-        <v>718.8</v>
+        <v>1828.5</v>
       </c>
       <c r="J31" t="n">
-        <v>799.47</v>
+        <v>789.9400000000001</v>
       </c>
       <c r="K31" t="n">
-        <v>-10.1</v>
+        <v>131.5</v>
       </c>
       <c r="L31" t="n">
-        <v>73.2</v>
+        <v>67.55</v>
       </c>
       <c r="M31" t="n">
-        <v>1.42</v>
+        <v>12.76</v>
       </c>
       <c r="N31" t="n">
-        <v>14160174</v>
+        <v>127606073</v>
       </c>
       <c r="O31" t="n">
-        <v>0</v>
+        <v>130033072</v>
       </c>
       <c r="P31" t="n">
-        <v>14160174</v>
+        <v>-2426999</v>
       </c>
       <c r="Q31" t="n">
-        <v>0</v>
+        <v>101.9</v>
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>Net Buying</t>
+          <t>Net Selling</t>
         </is>
       </c>
       <c r="S31" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T31" t="n">
+        <v>6</v>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>25-06-2026</t>
+        </is>
+      </c>
+      <c r="V31" t="n">
+        <v>0</v>
+      </c>
+      <c r="W31" t="n">
+        <v>3815</v>
+      </c>
+      <c r="X31" t="n">
+        <v>85.90000000000001</v>
+      </c>
+      <c r="Y31" t="n">
+        <v>42</v>
+      </c>
+      <c r="Z31" t="n">
+        <v>13</v>
+      </c>
+      <c r="AA31" t="n">
+        <v>22</v>
+      </c>
+      <c r="AB31" t="n">
+        <v>5.05</v>
+      </c>
+      <c r="AC31" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="AD31" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AE31" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF31" t="n">
+        <v>27</v>
+      </c>
+      <c r="AG31" t="n">
+        <v>1614.67</v>
+      </c>
+      <c r="AH31" t="n">
+        <v>1381.2</v>
+      </c>
+      <c r="AI31" t="n">
+        <v>108.1</v>
+      </c>
+      <c r="AJ31" t="n">
+        <v>789.9446136512771</v>
+      </c>
+      <c r="AK31" t="n">
+        <v>131.5</v>
+      </c>
+      <c r="AL31" t="inlineStr">
+        <is>
+          <t>Stale</t>
+        </is>
+      </c>
+      <c r="AM31" t="inlineStr">
+        <is>
+          <t>Stale Accumulation</t>
+        </is>
+      </c>
+      <c r="AN31" t="inlineStr">
+        <is>
+          <t>Late — Poor Entry</t>
+        </is>
+      </c>
+      <c r="AO31" t="inlineStr">
+        <is>
+          <t>25-06-2026</t>
+        </is>
+      </c>
+      <c r="AP31" t="inlineStr">
+        <is>
+          <t>25-06-2026</t>
+        </is>
+      </c>
+      <c r="AQ31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR31" t="n">
+        <v>88</v>
+      </c>
+      <c r="AS31" t="n">
+        <v>88</v>
+      </c>
+      <c r="AT31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX31" t="n">
+        <v>12</v>
+      </c>
+      <c r="AY31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC31" t="n">
+        <v>255212146</v>
+      </c>
+      <c r="BD31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH31" t="n">
         <v>4</v>
       </c>
-      <c r="U31" t="inlineStr">
-        <is>
-          <t>17-09-2026</t>
-        </is>
-      </c>
-      <c r="V31" t="n">
-        <v>0.195</v>
-      </c>
-      <c r="W31" t="n">
-        <v>728</v>
-      </c>
-      <c r="X31" t="n">
-        <v>13.2</v>
-      </c>
-      <c r="Y31" t="n">
-        <v>185</v>
-      </c>
-      <c r="Z31" t="n">
-        <v>11.55</v>
-      </c>
-      <c r="AA31" t="n">
-        <v>204</v>
-      </c>
-      <c r="AB31" t="n">
-        <v>6.84</v>
-      </c>
-      <c r="AC31" t="n">
-        <v>50.7</v>
-      </c>
-      <c r="AD31" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-      <c r="AE31" t="b">
-        <v>1</v>
-      </c>
-      <c r="AF31" t="n">
-        <v>16.07</v>
-      </c>
-      <c r="AG31" t="n">
-        <v>729.78</v>
-      </c>
-      <c r="AH31" t="inlineStr"/>
-      <c r="AI31" t="n">
-        <v>-20.9</v>
-      </c>
-      <c r="AJ31" t="n">
-        <v>799.4678184281843</v>
-      </c>
-      <c r="AK31" t="n">
-        <v>-10.1</v>
-      </c>
-      <c r="AL31" t="inlineStr">
-        <is>
-          <t>Fresh</t>
-        </is>
-      </c>
-      <c r="AM31" t="inlineStr">
-        <is>
-          <t>Confirmed Accumulation</t>
-        </is>
-      </c>
-      <c r="AN31" t="inlineStr">
-        <is>
-          <t>Confirmed Accumulation</t>
-        </is>
-      </c>
-      <c r="AO31" t="inlineStr">
-        <is>
-          <t>19-06-2026</t>
-        </is>
-      </c>
-      <c r="AP31" t="inlineStr">
-        <is>
-          <t>17-09-2026</t>
-        </is>
-      </c>
-      <c r="AQ31" t="n">
-        <v>90</v>
-      </c>
-      <c r="AR31" t="n">
-        <v>94</v>
-      </c>
-      <c r="AS31" t="n">
-        <v>4</v>
-      </c>
-      <c r="AT31" t="n">
-        <v>1</v>
-      </c>
-      <c r="AU31" t="n">
-        <v>1</v>
-      </c>
-      <c r="AV31" t="n">
-        <v>1</v>
-      </c>
-      <c r="AW31" t="n">
-        <v>1</v>
-      </c>
-      <c r="AX31" t="n">
-        <v>2</v>
-      </c>
-      <c r="AY31" t="n">
-        <v>1751854</v>
-      </c>
-      <c r="AZ31" t="n">
-        <v>1751854</v>
-      </c>
-      <c r="BA31" t="n">
-        <v>1751854</v>
-      </c>
-      <c r="BB31" t="n">
-        <v>1751854</v>
-      </c>
-      <c r="BC31" t="n">
-        <v>5375657</v>
-      </c>
-      <c r="BD31" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE31" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF31" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG31" t="n">
-        <v>0</v>
-      </c>
-      <c r="BH31" t="n">
-        <v>0</v>
-      </c>
       <c r="BI31" t="n">
         <v>0</v>
       </c>
@@ -7782,22 +7784,22 @@
         <v>0</v>
       </c>
       <c r="BM31" t="n">
-        <v>0</v>
+        <v>260066144</v>
       </c>
       <c r="BN31" t="n">
-        <v>1751854</v>
+        <v>0</v>
       </c>
       <c r="BO31" t="n">
-        <v>1751854</v>
+        <v>0</v>
       </c>
       <c r="BP31" t="n">
         <v>2</v>
       </c>
       <c r="BQ31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BR31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -8035,16 +8037,16 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>NPST</t>
+          <t>AMANTA</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>NETWORK PEOPLE SERVICES TECHNOLOGIES LIMITED</t>
+          <t>Amanta Healthcare Limited</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -8052,107 +8054,107 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F33" t="n">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="G33" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="H33" t="n">
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="I33" t="n">
-        <v>1828.5</v>
+        <v>189.95</v>
       </c>
       <c r="J33" t="n">
-        <v>789.9400000000001</v>
+        <v>149.98</v>
       </c>
       <c r="K33" t="n">
-        <v>131.5</v>
+        <v>26.7</v>
       </c>
       <c r="L33" t="n">
-        <v>67.55</v>
+        <v>63.56</v>
       </c>
       <c r="M33" t="n">
-        <v>12.76</v>
+        <v>0.24</v>
       </c>
       <c r="N33" t="n">
-        <v>127606073</v>
+        <v>2429680</v>
       </c>
       <c r="O33" t="n">
-        <v>130033072</v>
+        <v>0</v>
       </c>
       <c r="P33" t="n">
-        <v>-2426999</v>
+        <v>2429680</v>
       </c>
       <c r="Q33" t="n">
-        <v>101.9</v>
+        <v>0</v>
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>Net Selling</t>
+          <t>Net Buying</t>
         </is>
       </c>
       <c r="S33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T33" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="V33" t="n">
-        <v>0</v>
+        <v>0.033</v>
       </c>
       <c r="W33" t="n">
-        <v>3815</v>
+        <v>738</v>
       </c>
       <c r="X33" t="n">
-        <v>85.90000000000001</v>
+        <v>48.1</v>
       </c>
       <c r="Y33" t="n">
-        <v>42</v>
+        <v>7</v>
       </c>
       <c r="Z33" t="n">
-        <v>13</v>
+        <v>14.54</v>
       </c>
       <c r="AA33" t="n">
-        <v>22</v>
+        <v>-4</v>
       </c>
       <c r="AB33" t="n">
-        <v>5.05</v>
+        <v>0.85</v>
       </c>
       <c r="AC33" t="n">
-        <v>19.8</v>
+        <v>11.6</v>
       </c>
       <c r="AD33" t="n">
-        <v>0.03</v>
+        <v>1.11</v>
       </c>
       <c r="AE33" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF33" t="n">
-        <v>27</v>
+        <v>21.13</v>
       </c>
       <c r="AG33" t="n">
-        <v>1614.67</v>
+        <v>177.79</v>
       </c>
       <c r="AH33" t="n">
-        <v>1381.2</v>
+        <v>133.78</v>
       </c>
       <c r="AI33" t="n">
-        <v>108.1</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="AJ33" t="n">
-        <v>789.9446136512771</v>
+        <v>149.9802469135803</v>
       </c>
       <c r="AK33" t="n">
-        <v>131.5</v>
+        <v>26.7</v>
       </c>
       <c r="AL33" t="inlineStr">
         <is>
@@ -8171,22 +8173,22 @@
       </c>
       <c r="AO33" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="AP33" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="AQ33" t="n">
         <v>0</v>
       </c>
       <c r="AR33" t="n">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="AS33" t="n">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="AT33" t="n">
         <v>0</v>
@@ -8201,7 +8203,7 @@
         <v>0</v>
       </c>
       <c r="AX33" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="AY33" t="n">
         <v>0</v>
@@ -8216,7 +8218,7 @@
         <v>0</v>
       </c>
       <c r="BC33" t="n">
-        <v>255212146</v>
+        <v>0</v>
       </c>
       <c r="BD33" t="n">
         <v>0</v>
@@ -8231,7 +8233,7 @@
         <v>0</v>
       </c>
       <c r="BH33" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="BI33" t="n">
         <v>0</v>
@@ -8246,7 +8248,7 @@
         <v>0</v>
       </c>
       <c r="BM33" t="n">
-        <v>260066144</v>
+        <v>0</v>
       </c>
       <c r="BN33" t="n">
         <v>0</v>
@@ -8255,10 +8257,10 @@
         <v>0</v>
       </c>
       <c r="BP33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BQ33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BR33" t="n">
         <v>0</v>
@@ -8727,16 +8729,16 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>AMANTA</t>
+          <t>PLASTIBLEN</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Amanta Healthcare Limited</t>
+          <t>PLASTIBLENDS INDIA LIMITED</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -8744,107 +8746,107 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F36" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="G36" t="n">
         <v>21</v>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>-15</v>
       </c>
       <c r="I36" t="n">
-        <v>189.95</v>
+        <v>186.63</v>
       </c>
       <c r="J36" t="n">
-        <v>149.98</v>
+        <v>175.84</v>
       </c>
       <c r="K36" t="n">
-        <v>26.7</v>
+        <v>6.1</v>
       </c>
       <c r="L36" t="n">
-        <v>63.56</v>
+        <v>64.20999999999999</v>
       </c>
       <c r="M36" t="n">
-        <v>0.24</v>
+        <v>7.95</v>
       </c>
       <c r="N36" t="n">
-        <v>2429680</v>
+        <v>79549544</v>
       </c>
       <c r="O36" t="n">
-        <v>0</v>
+        <v>110497109</v>
       </c>
       <c r="P36" t="n">
-        <v>2429680</v>
+        <v>-30947565</v>
       </c>
       <c r="Q36" t="n">
-        <v>0</v>
+        <v>138.9</v>
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>Net Buying</t>
+          <t>Net Selling</t>
         </is>
       </c>
       <c r="S36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
       <c r="V36" t="n">
-        <v>0.033</v>
+        <v>0</v>
       </c>
       <c r="W36" t="n">
-        <v>738</v>
+        <v>485</v>
       </c>
       <c r="X36" t="n">
-        <v>48.1</v>
+        <v>11.4</v>
       </c>
       <c r="Y36" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Z36" t="n">
-        <v>14.54</v>
+        <v>22</v>
       </c>
       <c r="AA36" t="n">
-        <v>-4</v>
+        <v>36</v>
       </c>
       <c r="AB36" t="n">
-        <v>0.85</v>
+        <v>5.75</v>
       </c>
       <c r="AC36" t="n">
-        <v>11.6</v>
+        <v>10.7</v>
       </c>
       <c r="AD36" t="n">
-        <v>1.11</v>
+        <v>0.05</v>
       </c>
       <c r="AE36" t="b">
         <v>1</v>
       </c>
       <c r="AF36" t="n">
-        <v>21.13</v>
+        <v>10</v>
       </c>
       <c r="AG36" t="n">
-        <v>177.79</v>
+        <v>191.6</v>
       </c>
       <c r="AH36" t="n">
-        <v>133.78</v>
+        <v>166.91</v>
       </c>
       <c r="AI36" t="n">
-        <v>94.90000000000001</v>
+        <v>41.6</v>
       </c>
       <c r="AJ36" t="n">
-        <v>149.9802469135803</v>
+        <v>175.8389566755084</v>
       </c>
       <c r="AK36" t="n">
-        <v>26.7</v>
+        <v>6.1</v>
       </c>
       <c r="AL36" t="inlineStr">
         <is>
@@ -8863,22 +8865,22 @@
       </c>
       <c r="AO36" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
       <c r="AP36" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
       <c r="AQ36" t="n">
         <v>0</v>
       </c>
       <c r="AR36" t="n">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="AS36" t="n">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="AT36" t="n">
         <v>0</v>
@@ -8893,7 +8895,7 @@
         <v>0</v>
       </c>
       <c r="AX36" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AY36" t="n">
         <v>0</v>
@@ -8908,7 +8910,7 @@
         <v>0</v>
       </c>
       <c r="BC36" t="n">
-        <v>0</v>
+        <v>79549544</v>
       </c>
       <c r="BD36" t="n">
         <v>0</v>
@@ -8923,7 +8925,7 @@
         <v>0</v>
       </c>
       <c r="BH36" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="BI36" t="n">
         <v>0</v>
@@ -8938,7 +8940,7 @@
         <v>0</v>
       </c>
       <c r="BM36" t="n">
-        <v>0</v>
+        <v>110497109</v>
       </c>
       <c r="BN36" t="n">
         <v>0</v>
@@ -8947,10 +8949,10 @@
         <v>0</v>
       </c>
       <c r="BP36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BQ36" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BR36" t="n">
         <v>0</v>
@@ -8959,12 +8961,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>OMPOWER</t>
+          <t>VSTL</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Om Power Transmission Limited</t>
+          <t>VIBHOR STEEL TUBES LIMITED</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -8979,136 +8981,138 @@
         <v>5</v>
       </c>
       <c r="F37" t="n">
+        <v>9</v>
+      </c>
+      <c r="G37" t="n">
+        <v>13</v>
+      </c>
+      <c r="H37" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I37" t="n">
+        <v>113.54</v>
+      </c>
+      <c r="J37" t="n">
+        <v>111.01</v>
+      </c>
+      <c r="K37" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="L37" t="n">
+        <v>73.48</v>
+      </c>
+      <c r="M37" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="N37" t="n">
+        <v>4484713</v>
+      </c>
+      <c r="O37" t="n">
+        <v>0</v>
+      </c>
+      <c r="P37" t="n">
+        <v>4484713</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>0</v>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Net Buying</t>
+        </is>
+      </c>
+      <c r="S37" t="b">
+        <v>0</v>
+      </c>
+      <c r="T37" t="n">
+        <v>8</v>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>03-09-2026</t>
+        </is>
+      </c>
+      <c r="V37" t="n">
+        <v>0.209</v>
+      </c>
+      <c r="W37" t="n">
+        <v>215</v>
+      </c>
+      <c r="X37" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="Y37" t="n">
+        <v>21</v>
+      </c>
+      <c r="Z37" t="n">
+        <v>12.07</v>
+      </c>
+      <c r="AA37" t="n">
+        <v>-29</v>
+      </c>
+      <c r="AB37" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="AC37" t="n">
+        <v>7.92</v>
+      </c>
+      <c r="AD37" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="AE37" t="b">
+        <v>1</v>
+      </c>
+      <c r="AF37" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="AG37" t="n">
+        <v>112.01</v>
+      </c>
+      <c r="AH37" t="n">
+        <v>118.75</v>
+      </c>
+      <c r="AI37" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="AJ37" t="n">
+        <v>111.3431590909091</v>
+      </c>
+      <c r="AK37" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL37" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="AM37" t="inlineStr">
+        <is>
+          <t>Confirmed Accumulation</t>
+        </is>
+      </c>
+      <c r="AN37" t="inlineStr">
+        <is>
+          <t>Confirmed Accumulation</t>
+        </is>
+      </c>
+      <c r="AO37" t="inlineStr">
+        <is>
+          <t>17-08-2026</t>
+        </is>
+      </c>
+      <c r="AP37" t="inlineStr">
+        <is>
+          <t>03-09-2026</t>
+        </is>
+      </c>
+      <c r="AQ37" t="n">
         <v>17</v>
       </c>
-      <c r="G37" t="n">
-        <v>4</v>
-      </c>
-      <c r="H37" t="n">
-        <v>0</v>
-      </c>
-      <c r="I37" t="n">
-        <v>172.37</v>
-      </c>
-      <c r="J37" t="n">
-        <v>182.69</v>
-      </c>
-      <c r="K37" t="n">
-        <v>-5.6</v>
-      </c>
-      <c r="L37" t="n">
-        <v>69.05</v>
-      </c>
-      <c r="M37" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="N37" t="n">
-        <v>7447179</v>
-      </c>
-      <c r="O37" t="n">
-        <v>0</v>
-      </c>
-      <c r="P37" t="n">
-        <v>7447179</v>
-      </c>
-      <c r="Q37" t="n">
-        <v>0</v>
-      </c>
-      <c r="R37" t="inlineStr">
-        <is>
-          <t>Net Buying</t>
-        </is>
-      </c>
-      <c r="S37" t="b">
-        <v>0</v>
-      </c>
-      <c r="T37" t="n">
-        <v>3</v>
-      </c>
-      <c r="U37" t="inlineStr">
-        <is>
-          <t>24-06-2026</t>
-        </is>
-      </c>
-      <c r="V37" t="n">
-        <v>0.126</v>
-      </c>
-      <c r="W37" t="n">
-        <v>590</v>
-      </c>
-      <c r="X37" t="n">
-        <v>14</v>
-      </c>
-      <c r="Y37" t="n">
-        <v>61</v>
-      </c>
-      <c r="Z37" t="n">
-        <v>15</v>
-      </c>
-      <c r="AA37" t="n">
-        <v>82</v>
-      </c>
-      <c r="AB37" t="n">
-        <v>3.07</v>
-      </c>
-      <c r="AC37" t="n">
-        <v>42.7</v>
-      </c>
-      <c r="AD37" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="AE37" t="b">
-        <v>0</v>
-      </c>
-      <c r="AF37" t="n">
-        <v>12</v>
-      </c>
-      <c r="AG37" t="n">
-        <v>169.28</v>
-      </c>
-      <c r="AH37" t="inlineStr"/>
-      <c r="AI37" t="n">
-        <v>-10.9</v>
-      </c>
-      <c r="AJ37" t="n">
-        <v>182.6945759634963</v>
-      </c>
-      <c r="AK37" t="n">
-        <v>-5.7</v>
-      </c>
-      <c r="AL37" t="inlineStr">
-        <is>
-          <t>Stale</t>
-        </is>
-      </c>
-      <c r="AM37" t="inlineStr">
-        <is>
-          <t>Stale Accumulation</t>
-        </is>
-      </c>
-      <c r="AN37" t="inlineStr">
-        <is>
-          <t>Late — Poor Entry</t>
-        </is>
-      </c>
-      <c r="AO37" t="inlineStr">
-        <is>
-          <t>24-06-2026</t>
-        </is>
-      </c>
-      <c r="AP37" t="inlineStr">
-        <is>
-          <t>24-06-2026</t>
-        </is>
-      </c>
-      <c r="AQ37" t="n">
-        <v>0</v>
-      </c>
       <c r="AR37" t="n">
-        <v>89</v>
+        <v>35</v>
       </c>
       <c r="AS37" t="n">
-        <v>89</v>
+        <v>18</v>
       </c>
       <c r="AT37" t="n">
         <v>0</v>
@@ -9117,13 +9121,13 @@
         <v>0</v>
       </c>
       <c r="AV37" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="AW37" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="AX37" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="AY37" t="n">
         <v>0</v>
@@ -9132,13 +9136,13 @@
         <v>0</v>
       </c>
       <c r="BA37" t="n">
-        <v>0</v>
+        <v>3936339</v>
       </c>
       <c r="BB37" t="n">
-        <v>0</v>
+        <v>4899099</v>
       </c>
       <c r="BC37" t="n">
-        <v>7447179</v>
+        <v>4899099</v>
       </c>
       <c r="BD37" t="n">
         <v>0</v>
@@ -9174,10 +9178,10 @@
         <v>0</v>
       </c>
       <c r="BO37" t="n">
-        <v>0</v>
+        <v>3936339</v>
       </c>
       <c r="BP37" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="BQ37" t="n">
         <v>0</v>
@@ -9189,12 +9193,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>VSTL</t>
+          <t>OMPOWER</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>VIBHOR STEEL TUBES LIMITED</t>
+          <t>Om Power Transmission Limited</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -9209,37 +9213,37 @@
         <v>5</v>
       </c>
       <c r="F38" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="G38" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="H38" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I38" t="n">
-        <v>113.54</v>
+        <v>172.37</v>
       </c>
       <c r="J38" t="n">
-        <v>111.01</v>
+        <v>182.69</v>
       </c>
       <c r="K38" t="n">
-        <v>2.3</v>
+        <v>-5.6</v>
       </c>
       <c r="L38" t="n">
-        <v>73.48</v>
+        <v>69.05</v>
       </c>
       <c r="M38" t="n">
-        <v>0.45</v>
+        <v>0.74</v>
       </c>
       <c r="N38" t="n">
-        <v>4484713</v>
+        <v>7447179</v>
       </c>
       <c r="O38" t="n">
         <v>0</v>
       </c>
       <c r="P38" t="n">
-        <v>4484713</v>
+        <v>7447179</v>
       </c>
       <c r="Q38" t="n">
         <v>0</v>
@@ -9253,94 +9257,92 @@
         <v>0</v>
       </c>
       <c r="T38" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="U38" t="inlineStr">
         <is>
-          <t>03-09-2026</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="V38" t="n">
-        <v>0.209</v>
+        <v>0.126</v>
       </c>
       <c r="W38" t="n">
-        <v>215</v>
+        <v>590</v>
       </c>
       <c r="X38" t="n">
-        <v>25.6</v>
+        <v>14</v>
       </c>
       <c r="Y38" t="n">
-        <v>21</v>
+        <v>61</v>
       </c>
       <c r="Z38" t="n">
-        <v>12.07</v>
+        <v>15</v>
       </c>
       <c r="AA38" t="n">
-        <v>-29</v>
+        <v>82</v>
       </c>
       <c r="AB38" t="n">
-        <v>1.02</v>
+        <v>3.07</v>
       </c>
       <c r="AC38" t="n">
-        <v>7.92</v>
+        <v>42.7</v>
       </c>
       <c r="AD38" t="n">
-        <v>0.98</v>
+        <v>0.35</v>
       </c>
       <c r="AE38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF38" t="n">
-        <v>4.11</v>
+        <v>12</v>
       </c>
       <c r="AG38" t="n">
-        <v>112.01</v>
-      </c>
-      <c r="AH38" t="n">
-        <v>118.75</v>
-      </c>
+        <v>169.28</v>
+      </c>
+      <c r="AH38" t="inlineStr"/>
       <c r="AI38" t="n">
-        <v>5.2</v>
+        <v>-10.9</v>
       </c>
       <c r="AJ38" t="n">
-        <v>111.3431590909091</v>
+        <v>182.6945759634963</v>
       </c>
       <c r="AK38" t="n">
-        <v>2</v>
+        <v>-5.7</v>
       </c>
       <c r="AL38" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Stale</t>
         </is>
       </c>
       <c r="AM38" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Stale Accumulation</t>
         </is>
       </c>
       <c r="AN38" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Late — Poor Entry</t>
         </is>
       </c>
       <c r="AO38" t="inlineStr">
         <is>
-          <t>17-08-2026</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="AP38" t="inlineStr">
         <is>
-          <t>03-09-2026</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="AQ38" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="AR38" t="n">
-        <v>35</v>
+        <v>89</v>
       </c>
       <c r="AS38" t="n">
-        <v>18</v>
+        <v>89</v>
       </c>
       <c r="AT38" t="n">
         <v>0</v>
@@ -9349,13 +9351,13 @@
         <v>0</v>
       </c>
       <c r="AV38" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="AW38" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="AX38" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="AY38" t="n">
         <v>0</v>
@@ -9364,13 +9366,13 @@
         <v>0</v>
       </c>
       <c r="BA38" t="n">
-        <v>3936339</v>
+        <v>0</v>
       </c>
       <c r="BB38" t="n">
-        <v>4899099</v>
+        <v>0</v>
       </c>
       <c r="BC38" t="n">
-        <v>4899099</v>
+        <v>7447179</v>
       </c>
       <c r="BD38" t="n">
         <v>0</v>
@@ -9406,10 +9408,10 @@
         <v>0</v>
       </c>
       <c r="BO38" t="n">
-        <v>3936339</v>
+        <v>0</v>
       </c>
       <c r="BP38" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BQ38" t="n">
         <v>0</v>
@@ -9421,16 +9423,16 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>PLASTIBLEN</t>
+          <t>HEXAGON</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>PLASTIBLENDS INDIA LIMITED</t>
+          <t>HEXAGON NUTRITION LIMITED</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -9438,171 +9440,163 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F39" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="G39" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="H39" t="n">
-        <v>-15</v>
+        <v>0</v>
       </c>
       <c r="I39" t="n">
-        <v>186.63</v>
+        <v>66.26000000000001</v>
       </c>
       <c r="J39" t="n">
-        <v>175.84</v>
+        <v>64.48999999999999</v>
       </c>
       <c r="K39" t="n">
-        <v>6.1</v>
+        <v>2.7</v>
       </c>
       <c r="L39" t="n">
-        <v>64.20999999999999</v>
+        <v>64.29000000000001</v>
       </c>
       <c r="M39" t="n">
-        <v>7.95</v>
+        <v>0.57</v>
       </c>
       <c r="N39" t="n">
-        <v>79549544</v>
+        <v>5656038</v>
       </c>
       <c r="O39" t="n">
-        <v>110497109</v>
+        <v>0</v>
       </c>
       <c r="P39" t="n">
-        <v>-30947565</v>
+        <v>5656038</v>
       </c>
       <c r="Q39" t="n">
-        <v>138.9</v>
+        <v>0</v>
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>Net Selling</t>
+          <t>Net Buying</t>
         </is>
       </c>
       <c r="S39" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T39" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="U39" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>18-09-2026</t>
         </is>
       </c>
       <c r="V39" t="n">
-        <v>0</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="W39" t="n">
-        <v>485</v>
+        <v>814</v>
       </c>
       <c r="X39" t="n">
-        <v>11.4</v>
-      </c>
-      <c r="Y39" t="n">
-        <v>5</v>
-      </c>
+        <v>19.5</v>
+      </c>
+      <c r="Y39" t="inlineStr"/>
       <c r="Z39" t="n">
-        <v>22</v>
-      </c>
-      <c r="AA39" t="n">
-        <v>36</v>
-      </c>
+        <v>12.31</v>
+      </c>
+      <c r="AA39" t="inlineStr"/>
       <c r="AB39" t="n">
-        <v>5.75</v>
-      </c>
-      <c r="AC39" t="n">
-        <v>10.7</v>
-      </c>
+        <v>0.8</v>
+      </c>
+      <c r="AC39" t="inlineStr"/>
       <c r="AD39" t="n">
-        <v>0.05</v>
+        <v>0.11</v>
       </c>
       <c r="AE39" t="b">
         <v>1</v>
       </c>
       <c r="AF39" t="n">
-        <v>10</v>
+        <v>12.14</v>
       </c>
       <c r="AG39" t="n">
-        <v>191.6</v>
-      </c>
-      <c r="AH39" t="n">
-        <v>166.91</v>
-      </c>
+        <v>67.17</v>
+      </c>
+      <c r="AH39" t="inlineStr"/>
       <c r="AI39" t="n">
-        <v>41.6</v>
+        <v>30.8</v>
       </c>
       <c r="AJ39" t="n">
-        <v>175.8389566755084</v>
+        <v>64.33497045790251</v>
       </c>
       <c r="AK39" t="n">
-        <v>6.1</v>
+        <v>3</v>
       </c>
       <c r="AL39" t="inlineStr">
         <is>
-          <t>Stale</t>
+          <t>Fresh</t>
         </is>
       </c>
       <c r="AM39" t="inlineStr">
         <is>
-          <t>Stale Accumulation</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AN39" t="inlineStr">
         <is>
-          <t>Late — Poor Entry</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AO39" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>17-08-2026</t>
         </is>
       </c>
       <c r="AP39" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>18-09-2026</t>
         </is>
       </c>
       <c r="AQ39" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="AR39" t="n">
-        <v>88</v>
+        <v>35</v>
       </c>
       <c r="AS39" t="n">
-        <v>88</v>
+        <v>3</v>
       </c>
       <c r="AT39" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AU39" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AV39" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AW39" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="AX39" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="AY39" t="n">
-        <v>0</v>
+        <v>2601121</v>
       </c>
       <c r="AZ39" t="n">
-        <v>0</v>
+        <v>2601121</v>
       </c>
       <c r="BA39" t="n">
-        <v>0</v>
+        <v>2601121</v>
       </c>
       <c r="BB39" t="n">
-        <v>0</v>
+        <v>8710955</v>
       </c>
       <c r="BC39" t="n">
-        <v>79549544</v>
+        <v>8710955</v>
       </c>
       <c r="BD39" t="n">
         <v>0</v>
@@ -9617,48 +9611,48 @@
         <v>0</v>
       </c>
       <c r="BH39" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI39" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ39" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK39" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL39" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM39" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN39" t="n">
+        <v>2601121</v>
+      </c>
+      <c r="BO39" t="n">
+        <v>2601121</v>
+      </c>
+      <c r="BP39" t="n">
         <v>4</v>
       </c>
-      <c r="BI39" t="n">
-        <v>0</v>
-      </c>
-      <c r="BJ39" t="n">
-        <v>0</v>
-      </c>
-      <c r="BK39" t="n">
-        <v>0</v>
-      </c>
-      <c r="BL39" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM39" t="n">
-        <v>110497109</v>
-      </c>
-      <c r="BN39" t="n">
-        <v>0</v>
-      </c>
-      <c r="BO39" t="n">
-        <v>0</v>
-      </c>
-      <c r="BP39" t="n">
-        <v>2</v>
-      </c>
       <c r="BQ39" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BR39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>HEXAGON</t>
+          <t>VIVIANA</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>HEXAGON NUTRITION LIMITED</t>
+          <t>VIVIANA POWER TECH LIMITED</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -9670,40 +9664,40 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F40" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="G40" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H40" t="n">
         <v>0</v>
       </c>
       <c r="I40" t="n">
-        <v>66.26000000000001</v>
+        <v>718.8</v>
       </c>
       <c r="J40" t="n">
-        <v>64.48999999999999</v>
+        <v>782.6</v>
       </c>
       <c r="K40" t="n">
-        <v>2.7</v>
+        <v>-8.199999999999999</v>
       </c>
       <c r="L40" t="n">
-        <v>64.29000000000001</v>
+        <v>73.2</v>
       </c>
       <c r="M40" t="n">
-        <v>0.57</v>
+        <v>0.54</v>
       </c>
       <c r="N40" t="n">
-        <v>5656038</v>
+        <v>5375657</v>
       </c>
       <c r="O40" t="n">
         <v>0</v>
       </c>
       <c r="P40" t="n">
-        <v>5656038</v>
+        <v>5375657</v>
       </c>
       <c r="Q40" t="n">
         <v>0</v>
@@ -9717,52 +9711,58 @@
         <v>0</v>
       </c>
       <c r="T40" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="U40" t="inlineStr">
         <is>
-          <t>18-09-2026</t>
+          <t>17-09-2026</t>
         </is>
       </c>
       <c r="V40" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.074</v>
       </c>
       <c r="W40" t="n">
-        <v>814</v>
+        <v>728</v>
       </c>
       <c r="X40" t="n">
-        <v>19.5</v>
-      </c>
-      <c r="Y40" t="inlineStr"/>
+        <v>13.2</v>
+      </c>
+      <c r="Y40" t="n">
+        <v>185</v>
+      </c>
       <c r="Z40" t="n">
-        <v>12.31</v>
-      </c>
-      <c r="AA40" t="inlineStr"/>
+        <v>11.55</v>
+      </c>
+      <c r="AA40" t="n">
+        <v>204</v>
+      </c>
       <c r="AB40" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AC40" t="inlineStr"/>
+        <v>6.84</v>
+      </c>
+      <c r="AC40" t="n">
+        <v>50.7</v>
+      </c>
       <c r="AD40" t="n">
-        <v>0.11</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="AE40" t="b">
         <v>1</v>
       </c>
       <c r="AF40" t="n">
-        <v>12.14</v>
+        <v>16.07</v>
       </c>
       <c r="AG40" t="n">
-        <v>67.17</v>
+        <v>729.78</v>
       </c>
       <c r="AH40" t="inlineStr"/>
       <c r="AI40" t="n">
-        <v>30.8</v>
+        <v>-20.9</v>
       </c>
       <c r="AJ40" t="n">
-        <v>64.33497045790251</v>
+        <v>782.5967389721939</v>
       </c>
       <c r="AK40" t="n">
-        <v>3</v>
+        <v>-8.199999999999999</v>
       </c>
       <c r="AL40" t="inlineStr">
         <is>
@@ -9781,52 +9781,52 @@
       </c>
       <c r="AO40" t="inlineStr">
         <is>
-          <t>17-08-2026</t>
+          <t>29-06-2026</t>
         </is>
       </c>
       <c r="AP40" t="inlineStr">
         <is>
-          <t>18-09-2026</t>
+          <t>17-09-2026</t>
         </is>
       </c>
       <c r="AQ40" t="n">
-        <v>32</v>
+        <v>80</v>
       </c>
       <c r="AR40" t="n">
-        <v>35</v>
+        <v>84</v>
       </c>
       <c r="AS40" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AT40" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AU40" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AV40" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AW40" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AX40" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="AY40" t="n">
-        <v>2601121</v>
+        <v>1751854</v>
       </c>
       <c r="AZ40" t="n">
-        <v>2601121</v>
+        <v>1751854</v>
       </c>
       <c r="BA40" t="n">
-        <v>2601121</v>
+        <v>1751854</v>
       </c>
       <c r="BB40" t="n">
-        <v>8710955</v>
+        <v>1751854</v>
       </c>
       <c r="BC40" t="n">
-        <v>8710955</v>
+        <v>5375657</v>
       </c>
       <c r="BD40" t="n">
         <v>0</v>
@@ -9859,13 +9859,13 @@
         <v>0</v>
       </c>
       <c r="BN40" t="n">
-        <v>2601121</v>
+        <v>1751854</v>
       </c>
       <c r="BO40" t="n">
-        <v>2601121</v>
+        <v>1751854</v>
       </c>
       <c r="BP40" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="BQ40" t="n">
         <v>0</v>
@@ -11740,7 +11740,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -11748,7 +11748,7 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F49" t="n">
         <v>8</v>
@@ -11763,25 +11763,25 @@
         <v>81.64</v>
       </c>
       <c r="J49" t="n">
-        <v>92.05</v>
+        <v>91.22</v>
       </c>
       <c r="K49" t="n">
-        <v>-11.3</v>
+        <v>-10.5</v>
       </c>
       <c r="L49" t="n">
         <v>71.72</v>
       </c>
       <c r="M49" t="n">
-        <v>2.3</v>
+        <v>1.37</v>
       </c>
       <c r="N49" t="n">
-        <v>22971294</v>
+        <v>13682958</v>
       </c>
       <c r="O49" t="n">
         <v>0</v>
       </c>
       <c r="P49" t="n">
-        <v>22971294</v>
+        <v>13682958</v>
       </c>
       <c r="Q49" t="n">
         <v>0</v>
@@ -11795,7 +11795,7 @@
         <v>0</v>
       </c>
       <c r="T49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U49" t="inlineStr">
         <is>
@@ -11803,7 +11803,7 @@
         </is>
       </c>
       <c r="V49" t="n">
-        <v>0.136</v>
+        <v>0.081</v>
       </c>
       <c r="W49" t="n">
         <v>1692</v>
@@ -11845,10 +11845,10 @@
         <v>-46.7</v>
       </c>
       <c r="AJ49" t="n">
-        <v>91.73975462149539</v>
+        <v>91.21972</v>
       </c>
       <c r="AK49" t="n">
-        <v>-11</v>
+        <v>-10.5</v>
       </c>
       <c r="AL49" t="inlineStr">
         <is>
@@ -11867,7 +11867,7 @@
       </c>
       <c r="AO49" t="inlineStr">
         <is>
-          <t>17-06-2026</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="AP49" t="inlineStr">
@@ -11876,10 +11876,10 @@
         </is>
       </c>
       <c r="AQ49" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="AR49" t="n">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="AS49" t="n">
         <v>89</v>
@@ -13282,35 +13282,35 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>VIVIANA</t>
+          <t>NPST</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>VIVIANA POWER TECH LIMITED</t>
+          <t>NETWORK PEOPLE SERVICES TECHNOLOGIES LIMITED</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>718.8</v>
+        <v>1828.5</v>
       </c>
       <c r="D31" t="n">
-        <v>799.47</v>
+        <v>789.9400000000001</v>
       </c>
       <c r="E31" t="n">
-        <v>-10.1</v>
+        <v>131.5</v>
       </c>
       <c r="F31" t="n">
-        <v>73.2</v>
+        <v>67.55</v>
       </c>
       <c r="G31" t="n">
-        <v>1.42</v>
+        <v>12.76</v>
       </c>
       <c r="H31" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>17-09-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
     </row>
@@ -13352,35 +13352,35 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>NPST</t>
+          <t>AMANTA</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>NETWORK PEOPLE SERVICES TECHNOLOGIES LIMITED</t>
+          <t>Amanta Healthcare Limited</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1828.5</v>
+        <v>189.95</v>
       </c>
       <c r="D33" t="n">
-        <v>789.9400000000001</v>
+        <v>149.98</v>
       </c>
       <c r="E33" t="n">
-        <v>131.5</v>
+        <v>26.7</v>
       </c>
       <c r="F33" t="n">
-        <v>67.55</v>
+        <v>63.56</v>
       </c>
       <c r="G33" t="n">
-        <v>12.76</v>
+        <v>0.24</v>
       </c>
       <c r="H33" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
     </row>
@@ -13457,175 +13457,175 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>AMANTA</t>
+          <t>PLASTIBLEN</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Amanta Healthcare Limited</t>
+          <t>PLASTIBLENDS INDIA LIMITED</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>189.95</v>
+        <v>186.63</v>
       </c>
       <c r="D36" t="n">
-        <v>149.98</v>
+        <v>175.84</v>
       </c>
       <c r="E36" t="n">
-        <v>26.7</v>
+        <v>6.1</v>
       </c>
       <c r="F36" t="n">
-        <v>63.56</v>
+        <v>64.20999999999999</v>
       </c>
       <c r="G36" t="n">
-        <v>0.24</v>
+        <v>7.95</v>
       </c>
       <c r="H36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>OMPOWER</t>
+          <t>VSTL</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Om Power Transmission Limited</t>
+          <t>VIBHOR STEEL TUBES LIMITED</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>172.37</v>
+        <v>113.54</v>
       </c>
       <c r="D37" t="n">
-        <v>182.69</v>
+        <v>111.01</v>
       </c>
       <c r="E37" t="n">
-        <v>-5.6</v>
+        <v>2.3</v>
       </c>
       <c r="F37" t="n">
-        <v>69.05</v>
+        <v>73.48</v>
       </c>
       <c r="G37" t="n">
-        <v>0.74</v>
+        <v>0.45</v>
       </c>
       <c r="H37" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>24-06-2026</t>
+          <t>03-09-2026</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>VSTL</t>
+          <t>OMPOWER</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>VIBHOR STEEL TUBES LIMITED</t>
+          <t>Om Power Transmission Limited</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>113.54</v>
+        <v>172.37</v>
       </c>
       <c r="D38" t="n">
-        <v>111.01</v>
+        <v>182.69</v>
       </c>
       <c r="E38" t="n">
-        <v>2.3</v>
+        <v>-5.6</v>
       </c>
       <c r="F38" t="n">
-        <v>73.48</v>
+        <v>69.05</v>
       </c>
       <c r="G38" t="n">
-        <v>0.45</v>
+        <v>0.74</v>
       </c>
       <c r="H38" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>03-09-2026</t>
+          <t>24-06-2026</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>PLASTIBLEN</t>
+          <t>HEXAGON</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>PLASTIBLENDS INDIA LIMITED</t>
+          <t>HEXAGON NUTRITION LIMITED</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>186.63</v>
+        <v>66.26000000000001</v>
       </c>
       <c r="D39" t="n">
-        <v>175.84</v>
+        <v>64.48999999999999</v>
       </c>
       <c r="E39" t="n">
-        <v>6.1</v>
+        <v>2.7</v>
       </c>
       <c r="F39" t="n">
-        <v>64.20999999999999</v>
+        <v>64.29000000000001</v>
       </c>
       <c r="G39" t="n">
-        <v>7.95</v>
+        <v>0.57</v>
       </c>
       <c r="H39" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>18-09-2026</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>HEXAGON</t>
+          <t>VIVIANA</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>HEXAGON NUTRITION LIMITED</t>
+          <t>VIVIANA POWER TECH LIMITED</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>66.26000000000001</v>
+        <v>718.8</v>
       </c>
       <c r="D40" t="n">
-        <v>64.48999999999999</v>
+        <v>782.6</v>
       </c>
       <c r="E40" t="n">
-        <v>2.7</v>
+        <v>-8.199999999999999</v>
       </c>
       <c r="F40" t="n">
-        <v>64.29000000000001</v>
+        <v>73.2</v>
       </c>
       <c r="G40" t="n">
-        <v>0.57</v>
+        <v>0.54</v>
       </c>
       <c r="H40" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>18-09-2026</t>
+          <t>17-09-2026</t>
         </is>
       </c>
     </row>
@@ -13924,19 +13924,19 @@
         <v>81.64</v>
       </c>
       <c r="D49" t="n">
-        <v>92.05</v>
+        <v>91.22</v>
       </c>
       <c r="E49" t="n">
-        <v>-11.3</v>
+        <v>-10.5</v>
       </c>
       <c r="F49" t="n">
         <v>71.72</v>
       </c>
       <c r="G49" t="n">
-        <v>2.3</v>
+        <v>1.37</v>
       </c>
       <c r="H49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
@@ -14012,7 +14012,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3">
@@ -14022,7 +14022,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">

</xml_diff>